<commit_message>
Add datasets, load_data.sql, and processed files
</commit_message>
<xml_diff>
--- a/data/raw/fmcsa_carrier_compliance.xlsx
+++ b/data/raw/fmcsa_carrier_compliance.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/atharvabhalilkar/Documents/freight-analytics/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5AD06CE-1971-A744-9640-6E4EFB18557E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CF3BF73-7B1E-164A-9885-1F0DA2D0545D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="660" windowWidth="28040" windowHeight="16940" xr2:uid="{246BB801-D6DE-1A4A-B473-22663E91EF72}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{246BB801-D6DE-1A4A-B473-22663E91EF72}"/>
   </bookViews>
   <sheets>
     <sheet name="fmcsa_carrier_compliance" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="62">
   <si>
     <t>carrier_name</t>
   </si>
@@ -1154,6 +1154,9 @@
       <c r="B4">
         <v>100003</v>
       </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
       <c r="D4" t="s">
         <v>11</v>
       </c>

</xml_diff>